<commit_message>
Update BugReport and add Screenshots
</commit_message>
<xml_diff>
--- a/06_Bug_Report/BugReport_Login.xlsx
+++ b/06_Bug_Report/BugReport_Login.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Manual-Tester-Portfolio\06_Bug_Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6089FD3-0BD5-4F70-8BF9-07E46F24BFCB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE66BDC4-5D64-4110-A365-0F6BBCEE3E7F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F2B45D61-9316-4E3F-8DBD-24FA297E3A0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F2B45D61-9316-4E3F-8DBD-24FA297E3A0E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Report Login" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="53">
   <si>
     <t>BUG REPORT - LOGIN MODULE</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>The user is required to log in again.</t>
+  </si>
+  <si>
+    <t>Closed</t>
   </si>
 </sst>
 </file>
@@ -315,20 +318,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FFC00000"/>
@@ -474,295 +477,6 @@
       <fill>
         <patternFill>
           <bgColor theme="6" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF600000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF4343"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF552579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDEC8EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF552579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDEC8EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF552579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDEC8EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF8B8B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7171"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1107,21 +821,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
     </row>
     <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1195,8 +909,8 @@
       <c r="J4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="8" t="s">
-        <v>29</v>
+      <c r="K4" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>28</v>
@@ -1234,8 +948,8 @@
       <c r="J5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="8" t="s">
-        <v>29</v>
+      <c r="K5" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>28</v>
@@ -1273,8 +987,8 @@
       <c r="J6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="8" t="s">
-        <v>29</v>
+      <c r="K6" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>28</v>
@@ -1312,8 +1026,8 @@
       <c r="J7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="8" t="s">
-        <v>29</v>
+      <c r="K7" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L7" s="3" t="s">
         <v>28</v>
@@ -1351,8 +1065,8 @@
       <c r="J8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="8" t="s">
-        <v>29</v>
+      <c r="K8" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>28</v>
@@ -1378,7 +1092,7 @@
       <c r="F9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>50</v>
       </c>
       <c r="H9" s="6" t="s">
@@ -1390,8 +1104,8 @@
       <c r="J9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="K9" s="8" t="s">
-        <v>29</v>
+      <c r="K9" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>28</v>
@@ -1484,7 +1198,7 @@
       <c r="D3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1501,7 +1215,7 @@
       <c r="D4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1518,7 +1232,7 @@
       <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1535,7 +1249,7 @@
       <c r="D6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1552,7 +1266,7 @@
       <c r="D7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1569,7 +1283,7 @@
       <c r="D8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>